<commit_message>
feat: creating docker file and compose
</commit_message>
<xml_diff>
--- a/ATDD.xlsx
+++ b/ATDD.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devops\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9444849349692f87/Documentos/workspace/Projects/ATDD_SpringBoot_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBF7E38-7348-459E-9445-B1BC30669AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{6CBF7E38-7348-459E-9445-B1BC30669AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A54AE80-C460-47A2-B451-C6140DD6331F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="240" windowWidth="29040" windowHeight="16080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pb" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="74">
   <si>
     <t>PRODUCT BACKLOG</t>
   </si>
@@ -489,12 +489,57 @@
   <si>
     <t>E a promoção não deve ser aplicada novamente</t>
   </si>
+  <si>
+    <t>Dado um aluno que teve o plano atualizado automaticamente para Premium</t>
+  </si>
+  <si>
+    <t>Quando o aluno acessa a área de benefícios exclusivos da plataforma</t>
+  </si>
+  <si>
+    <t>Então o sistema deve conceder acesso completo aos benefícios, sem exigir qualquer solicitação manual</t>
+  </si>
+  <si>
+    <t>"@Test
+public void devePromoverParaPremiumAoConquistarDecimoSegundoCurso() {
+var aluno = new Aluno("Nathan", 11, "basico");
+}"</t>
+  </si>
+  <si>
+    <t>"@Test
+public void deveManterPlanoBasicoComMenosDe12Cursos() {
+var aluno = new Aluno("Nathan", 10, "basico");
+}"</t>
+  </si>
+  <si>
+    <t>"@Test
+public void deveLiberarBeneficiosAutomaticamenteAoTornarSePremium() {
+var aluno = new Aluno("Nathan", 11, "basico");
+}"</t>
+  </si>
+  <si>
+    <t>"@Test
+public void naoDeveLiberarBeneficiosSemAtingirPremium() {
+var aluno = new Aluno("Nathan", 10, "basico");
+}"</t>
+  </si>
+  <si>
+    <t>aluno.conquistarCurso();</t>
+  </si>
+  <si>
+    <t>assertEquals("premium", aluno.getPlano());</t>
+  </si>
+  <si>
+    <t>assertTrue(aluno.beneficiosLiberadosSemSolicitacao());</t>
+  </si>
+  <si>
+    <t>assertFalse(aluno.beneficiosLiberadosSemSolicitacao());</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -586,6 +631,11 @@
     <font>
       <sz val="36"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -762,7 +812,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -808,14 +858,32 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -850,29 +918,23 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1093,7 +1155,7 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="7.28515625" customWidth="1"/>
-    <col min="2" max="2" width="41.5703125" style="43" customWidth="1"/>
+    <col min="2" max="2" width="41.5703125" style="25" customWidth="1"/>
     <col min="3" max="3" width="62.28515625" customWidth="1"/>
     <col min="4" max="4" width="65.28515625" customWidth="1"/>
     <col min="5" max="5" width="56.28515625" customWidth="1"/>
@@ -1115,85 +1177,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="55.5" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="23"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="F1" s="1"/>
-      <c r="G1" s="27" t="s">
+      <c r="G1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="23"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="30"/>
       <c r="M1" s="1"/>
-      <c r="N1" s="28" t="s">
+      <c r="N1" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="23"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="30"/>
     </row>
     <row r="2" spans="1:19" ht="26.25" customHeight="1">
-      <c r="A2" s="29"/>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="31"/>
+      <c r="A2" s="35"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="36"/>
+      <c r="P2" s="36"/>
+      <c r="Q2" s="36"/>
+      <c r="R2" s="36"/>
+      <c r="S2" s="37"/>
     </row>
     <row r="3" spans="1:19" ht="36" customHeight="1">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="32" t="s">
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="32" t="s">
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="23"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="30"/>
     </row>
     <row r="4" spans="1:19" ht="66" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="22" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -1205,7 +1267,7 @@
       <c r="E4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="34"/>
+      <c r="F4" s="40"/>
       <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1224,203 +1286,233 @@
       <c r="L4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M4" s="34"/>
+      <c r="M4" s="40"/>
       <c r="N4" s="3" t="s">
         <v>15</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="38" t="s">
+      <c r="P4" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="23"/>
+      <c r="Q4" s="29"/>
+      <c r="R4" s="29"/>
+      <c r="S4" s="30"/>
     </row>
     <row r="5" spans="1:19" ht="370.5" customHeight="1">
       <c r="A5" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="39" t="s">
+      <c r="E5" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="34"/>
-      <c r="G5" s="45" t="s">
+      <c r="F5" s="40"/>
+      <c r="G5" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="H5" s="45" t="s">
+      <c r="H5" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="I5" s="45" t="s">
+      <c r="I5" s="27" t="s">
         <v>53</v>
       </c>
       <c r="J5" s="7"/>
-      <c r="K5" s="45" t="s">
+      <c r="K5" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="L5" s="46"/>
-      <c r="M5" s="34"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-      <c r="P5" s="25"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="23"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="40"/>
+      <c r="N5" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="O5" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="P5" s="45" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q5" s="46"/>
+      <c r="R5" s="46"/>
+      <c r="S5" s="47"/>
     </row>
     <row r="6" spans="1:19" ht="279">
       <c r="A6" s="9"/>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="39" t="s">
+      <c r="E6" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="34"/>
-      <c r="G6" s="44" t="s">
+      <c r="F6" s="40"/>
+      <c r="G6" s="26" t="s">
         <v>55</v>
       </c>
       <c r="H6" s="6"/>
-      <c r="I6" s="44" t="s">
+      <c r="I6" s="26" t="s">
         <v>56</v>
       </c>
       <c r="J6" s="6"/>
-      <c r="K6" s="44" t="s">
+      <c r="K6" s="26" t="s">
         <v>57</v>
       </c>
       <c r="L6" s="10"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="25"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="23"/>
+      <c r="M6" s="40"/>
+      <c r="N6" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="O6" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="P6" s="45" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q6" s="46"/>
+      <c r="R6" s="46"/>
+      <c r="S6" s="47"/>
     </row>
-    <row r="7" spans="1:19" ht="409.5">
+    <row r="7" spans="1:19" ht="279">
       <c r="A7" s="9"/>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="D7" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="39" t="s">
+      <c r="E7" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="F7" s="34"/>
-      <c r="G7" s="44" t="s">
+      <c r="F7" s="40"/>
+      <c r="G7" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="44" t="s">
+      <c r="H7" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="I7" s="44" t="s">
+      <c r="I7" s="26" t="s">
         <v>60</v>
       </c>
       <c r="J7" s="6"/>
-      <c r="K7" s="44" t="s">
+      <c r="K7" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="L7" s="44" t="s">
+      <c r="L7" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="M7" s="34"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="23"/>
+      <c r="M7" s="40"/>
+      <c r="N7" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="O7" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="P7" s="48" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q7" s="46"/>
+      <c r="R7" s="46"/>
+      <c r="S7" s="47"/>
     </row>
-    <row r="8" spans="1:19" ht="362.25" customHeight="1">
+    <row r="8" spans="1:19" ht="409.6" customHeight="1">
       <c r="A8" s="9"/>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="C8" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="39" t="s">
+      <c r="E8" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="34"/>
-      <c r="G8" s="6"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="26" t="s">
+        <v>63</v>
+      </c>
       <c r="H8" s="11"/>
-      <c r="I8" s="6"/>
+      <c r="I8" s="26" t="s">
+        <v>64</v>
+      </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="6"/>
+      <c r="K8" s="26" t="s">
+        <v>65</v>
+      </c>
       <c r="L8" s="11"/>
-      <c r="M8" s="34"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="24"/>
-      <c r="Q8" s="22"/>
-      <c r="R8" s="22"/>
-      <c r="S8" s="23"/>
+      <c r="M8" s="40"/>
+      <c r="N8" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="O8" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="P8" s="45" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q8" s="49"/>
+      <c r="R8" s="49"/>
+      <c r="S8" s="50"/>
     </row>
     <row r="9" spans="1:19" ht="355.5" customHeight="1">
       <c r="A9" s="9"/>
-      <c r="B9" s="42"/>
+      <c r="B9" s="24"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
-      <c r="F9" s="34"/>
+      <c r="F9" s="40"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="L9" s="11"/>
-      <c r="M9" s="34"/>
+      <c r="M9" s="40"/>
       <c r="N9" s="6"/>
       <c r="O9" s="6"/>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="22"/>
-      <c r="S9" s="23"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="29"/>
+      <c r="R9" s="29"/>
+      <c r="S9" s="30"/>
     </row>
     <row r="10" spans="1:19" ht="201" hidden="1" customHeight="1">
       <c r="A10" s="9"/>
-      <c r="B10" s="42"/>
+      <c r="B10" s="24"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
-      <c r="F10" s="35"/>
+      <c r="F10" s="41"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="9"/>
       <c r="L10" s="9"/>
-      <c r="M10" s="35"/>
+      <c r="M10" s="41"/>
       <c r="N10" s="9"/>
       <c r="O10" s="9"/>
-      <c r="P10" s="37"/>
-      <c r="Q10" s="22"/>
-      <c r="R10" s="22"/>
-      <c r="S10" s="23"/>
+      <c r="P10" s="43"/>
+      <c r="Q10" s="29"/>
+      <c r="R10" s="29"/>
+      <c r="S10" s="30"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>

</xml_diff>